<commit_message>
feat: updating project with separate student_name to first_name and last_name
</commit_message>
<xml_diff>
--- a/database-final.xlsx
+++ b/database-final.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="48">
   <si>
     <t>table:</t>
   </si>
@@ -31,7 +31,10 @@
     <t>id_student, PK</t>
   </si>
   <si>
-    <t>name_student</t>
+    <t>first_name</t>
+  </si>
+  <si>
+    <t>last_name</t>
   </si>
   <si>
     <t>classroom, FK</t>
@@ -49,7 +52,10 @@
     <t>course, PK</t>
   </si>
   <si>
-    <t>Ana Martínez</t>
+    <t>Ana</t>
+  </si>
+  <si>
+    <t>Martínez</t>
   </si>
   <si>
     <t>A101</t>
@@ -61,7 +67,10 @@
     <t>HTML</t>
   </si>
   <si>
-    <t>Luis Fernández</t>
+    <t xml:space="preserve">Luis </t>
+  </si>
+  <si>
+    <t>Fernández</t>
   </si>
   <si>
     <t>A102</t>
@@ -73,7 +82,10 @@
     <t>CSS</t>
   </si>
   <si>
-    <t>Carla Gómez</t>
+    <t xml:space="preserve">Carla </t>
+  </si>
+  <si>
+    <t>Gómez</t>
   </si>
   <si>
     <t>A103</t>
@@ -85,50 +97,71 @@
     <t>JavaScript</t>
   </si>
   <si>
-    <t>Diego López</t>
+    <t xml:space="preserve">Diego </t>
+  </si>
+  <si>
+    <t>López</t>
   </si>
   <si>
     <t>Java</t>
   </si>
   <si>
-    <t>Marta Sánchez</t>
+    <t xml:space="preserve">Marta </t>
+  </si>
+  <si>
+    <t>Sánchez</t>
   </si>
   <si>
     <t>Spring Framework</t>
   </si>
   <si>
-    <t>Javier Torres</t>
+    <t xml:space="preserve">Javier </t>
+  </si>
+  <si>
+    <t>Torres</t>
   </si>
   <si>
     <t>SQL</t>
   </si>
   <si>
-    <t>Laura Ruiz</t>
+    <t xml:space="preserve">Laura </t>
+  </si>
+  <si>
+    <t>Ruiz</t>
   </si>
   <si>
     <t>Kotlin</t>
   </si>
   <si>
-    <t>Pablo Ramírez</t>
+    <t xml:space="preserve">Pablo </t>
+  </si>
+  <si>
+    <t>Ramírez</t>
   </si>
   <si>
     <t>Swift</t>
   </si>
   <si>
-    <t>Sofía Navarro</t>
+    <t xml:space="preserve">Sofía </t>
+  </si>
+  <si>
+    <t>Navarro</t>
   </si>
   <si>
     <t>Dart</t>
   </si>
   <si>
-    <t>Tomás Ortega</t>
+    <t xml:space="preserve">Tomás </t>
+  </si>
+  <si>
+    <t>Ortega</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -160,6 +193,11 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -233,7 +271,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -258,6 +296,9 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -268,6 +309,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="8" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -484,16 +528,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="15.38"/>
     <col customWidth="1" min="2" max="2" width="19.13"/>
-    <col customWidth="1" min="3" max="3" width="15.63"/>
-    <col customWidth="1" min="5" max="5" width="15.38"/>
-    <col customWidth="1" min="6" max="6" width="25.88"/>
-    <col customWidth="1" min="8" max="8" width="19.38"/>
-    <col customWidth="1" min="9" max="9" width="33.13"/>
+    <col customWidth="1" min="3" max="4" width="15.63"/>
+    <col customWidth="1" min="6" max="6" width="15.38"/>
+    <col customWidth="1" min="7" max="7" width="25.88"/>
+    <col customWidth="1" min="9" max="9" width="19.38"/>
+    <col customWidth="1" min="10" max="10" width="33.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,20 +549,21 @@
         <v>1</v>
       </c>
       <c r="C1" s="2"/>
-      <c r="E1" s="1" t="s">
+      <c r="D1" s="2"/>
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2"/>
+      <c r="I1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
@@ -529,17 +575,20 @@
       <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="G3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="3" t="s">
         <v>11</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -547,22 +596,25 @@
         <v>1.0</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" s="8" t="s">
+      <c r="D4" s="9" t="s">
         <v>15</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -570,22 +622,25 @@
         <v>2.0</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" s="8" t="s">
         <v>19</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -593,22 +648,25 @@
         <v>3.0</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>23</v>
+        <v>25</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +674,19 @@
         <v>4.0</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="I7" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>25</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8">
@@ -633,16 +694,19 @@
         <v>5.0</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>27</v>
+        <v>32</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="9">
@@ -650,16 +714,19 @@
         <v>6.0</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>29</v>
+        <v>35</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="10">
@@ -667,16 +734,19 @@
         <v>7.0</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>31</v>
+        <v>38</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="11">
@@ -684,16 +754,19 @@
         <v>8.0</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>33</v>
+        <v>41</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="12">
@@ -701,30 +774,36 @@
         <v>9.0</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>21</v>
+        <v>44</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>35</v>
+        <v>25</v>
+      </c>
+      <c r="J12" s="11" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9">
+      <c r="A13" s="10">
         <v>10.0</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" s="7"/>
+      <c r="B13" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7"/>
@@ -755,6 +834,9 @@
       <c r="B28" s="7"/>
     </row>
   </sheetData>
+  <printOptions gridLines="1" horizontalCentered="1"/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup fitToHeight="0" paperSize="9" cellComments="atEnd" orientation="landscape" pageOrder="overThenDown"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>